<commit_message>
Update weekly WBS and gantt charts
</commit_message>
<xml_diff>
--- a/design/gantt/autofollowshoppingcart-day-gantt.xlsx
+++ b/design/gantt/autofollowshoppingcart-day-gantt.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务清单" sheetId="1" r:id="R5a94576d94ad478e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="日甘特图" sheetId="2" r:id="R0de779d335384df6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务清单" sheetId="1" r:id="R3abb940170a24fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="日甘特图" sheetId="2" r:id="R6cc0ed1f1f1044fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -154,12 +154,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE0E7FF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFA21CAF"/>
+        <x:fgColor rgb="FF374151"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -174,6 +169,11 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFA21CAF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF3F4F6"/>
       </x:patternFill>
     </x:fill>
@@ -184,12 +184,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFAE8FF"/>
+        <x:fgColor rgb="FFE0E7FF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF374151"/>
+        <x:fgColor rgb="FFFAE8FF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -368,6 +368,12 @@
     <x:xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
@@ -412,12 +418,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -473,14 +473,14 @@
     <x:xf numFmtId="201" fontId="9" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="10" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="10" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="10" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="10" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="10" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="10" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="8" fillId="23" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -489,7 +489,7 @@
     <x:xf numFmtId="201" fontId="9" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="10" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="10" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -508,10 +508,10 @@
     <x:xf numFmtId="201" fontId="0" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="201" fontId="9" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="8" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="10" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -800,7 +800,7 @@
         <x:v>T01</x:v>
       </x:c>
       <x:c r="B4" s="12" t="str">
-        <x:v>需求收口与关键指标确定</x:v>
+        <x:v>需求收口与首版边界确认</x:v>
       </x:c>
       <x:c r="C4" s="14" t="str">
         <x:v>成员 A / C</x:v>
@@ -818,15 +818,15 @@
         <x:v>项目规划</x:v>
       </x:c>
       <x:c r="H4" s="12" t="str">
-        <x:v>需求与指标口径定稿；对齐场景、功能边界和验收指标</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+        <x:v>需求与验收口径；明确 OpenBot + Android + ESP32/MCU + 底盘主线，不引入 SLAM/服务器主脑</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>T02</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>WBS、分工与物料清单初版</x:v>
+        <x:v>WBS、分工、BOM 初版</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
         <x:v>成员 C</x:v>
@@ -844,44 +844,44 @@
         <x:v>项目规划</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
-        <x:v>WBS、分工、BOM 初稿；建立项目管理主文档</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+        <x:v>WBS、分工、采购清单；完成首版任务拆解和核心物资采购口径</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
         <x:v>T03</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>方案 PPT 与汇报材料准备</x:v>
-      </x:c>
-      <x:c r="C6" s="14" t="str">
-        <x:v>成员 A / C</x:v>
+        <x:v>OpenBot App 环境与源码梳理</x:v>
+      </x:c>
+      <x:c r="C6" s="19" t="str">
+        <x:v>成员 A</x:v>
       </x:c>
       <x:c r="D6" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="13" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="13" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G6" s="17" t="str">
-        <x:v>项目规划</x:v>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G6" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="H6" s="12" t="str">
-        <x:v>方案 PPT 初版；用于第 1 周阶段汇报</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+        <x:v>OpenBot 上位机分析；确认 Android 手机作为上位机主脑</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
         <x:v>T04</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>OpenBot App 环境搭建与编译</x:v>
-      </x:c>
-      <x:c r="C7" s="19" t="str">
-        <x:v>成员 A</x:v>
+        <x:v>下位机方案与 AT8236 风险分析</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="str">
+        <x:v>成员 B</x:v>
       </x:c>
       <x:c r="D7" s="13" t="n">
         <x:v>1</x:v>
@@ -892,11 +892,11 @@
       <x:c r="F7" s="13" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G7" s="22" t="str">
-        <x:v>上位机</x:v>
+      <x:c r="G7" s="26" t="str">
+        <x:v>下位机</x:v>
       </x:c>
       <x:c r="H7" s="12" t="str">
-        <x:v>可运行 OpenBot App；记录构建环境和依赖版本</x:v>
+        <x:v>AT8236/ESP32 接口说明；确认 UART/I2C、驱动板、编码器和安全保护风险</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -904,25 +904,25 @@
         <x:v>T05</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>MCU 环境搭建与固件烧录</x:v>
-      </x:c>
-      <x:c r="C8" s="23" t="str">
-        <x:v>成员 B</x:v>
+        <x:v>底盘、电机、电池、驱动板采购</x:v>
+      </x:c>
+      <x:c r="C8" s="27" t="str">
+        <x:v>成员 B / C</x:v>
       </x:c>
       <x:c r="D8" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E8" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F8" s="13" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G8" s="26" t="str">
-        <x:v>下位机</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G8" s="30" t="str">
+        <x:v>硬件</x:v>
       </x:c>
       <x:c r="H8" s="12" t="str">
-        <x:v>可运行基础固件；打通 Arduino Nano 或 ESP32 基础控制</x:v>
+        <x:v>核心硬件到货/采购记录；覆盖麦轮底盘、AT8236、ESP32、12V 电池</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -930,224 +930,224 @@
         <x:v>T06</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>底盘、电机、电源到货检查</x:v>
-      </x:c>
-      <x:c r="C9" s="27" t="str">
-        <x:v>成员 B / C</x:v>
+        <x:v>方案 PPT 与第 1 周材料</x:v>
+      </x:c>
+      <x:c r="C9" s="14" t="str">
+        <x:v>成员 A / C</x:v>
       </x:c>
       <x:c r="D9" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E9" s="13" t="n">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F9" s="13" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G9" s="30" t="str">
-        <x:v>硬件</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G9" s="33" t="str">
+        <x:v>交付</x:v>
       </x:c>
       <x:c r="H9" s="12" t="str">
-        <x:v>到货验收记录；核对型号、接口和供电需求</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+        <x:v>第 1 周周志与汇报材料；形成第一轮课程交付材料</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
         <x:v>T07</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>手机与下位机串口通信打通</x:v>
-      </x:c>
-      <x:c r="C10" s="31" t="str">
-        <x:v>成员 B / A</x:v>
+        <x:v>Human Cart Simulator 主流程</x:v>
+      </x:c>
+      <x:c r="C10" s="19" t="str">
+        <x:v>成员 A</x:v>
       </x:c>
       <x:c r="D10" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E10" s="13" t="n">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F10" s="13" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G10" s="26" t="str">
-        <x:v>下位机</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G10" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="H10" s="12" t="str">
-        <x:v>通信链路可用；保留串口日志和异常记录</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+        <x:v>目标初始化与状态机；完成目标采集、截图确认、重识别、LOST/SEARCH/STOP 主链路</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
         <x:v>T08</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>底盘装配与基础运动联调</x:v>
-      </x:c>
-      <x:c r="C11" s="23" t="str">
-        <x:v>成员 B</x:v>
+        <x:v>距离控制图像伺服</x:v>
+      </x:c>
+      <x:c r="C11" s="19" t="str">
+        <x:v>成员 A</x:v>
       </x:c>
       <x:c r="D11" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E11" s="13" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F11" s="13" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G11" s="30" t="str">
-        <x:v>硬件</x:v>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="H11" s="12" t="str">
-        <x:v>底盘可稳定运动；完成前进、后退、转向、停车</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+        <x:v>DistanceState 距离控制；初始化 setpoint + height/area/bottom_shift，UNKNOWN 时停车</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
         <x:v>T09</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>手机支架与视角固定</x:v>
-      </x:c>
-      <x:c r="C12" s="18" t="str">
-        <x:v>成员 C</x:v>
+        <x:v>ReID PC 实验与 gallery 策略</x:v>
+      </x:c>
+      <x:c r="C12" s="19" t="str">
+        <x:v>成员 A</x:v>
       </x:c>
       <x:c r="D12" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E12" s="13" t="n">
-        <x:v>6</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F12" s="13" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G12" s="34" t="str">
-        <x:v>结构</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
-        <x:v>支架固定完成；保证画面稳定、视角合理</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+        <x:v>ReID 复测脚本与结论；osnet_x0_25 + diverse gallery(k=8)，ReID 只作身份置信辅助</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
         <x:v>T10</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>手动遥控测试与记录</x:v>
-      </x:c>
-      <x:c r="C13" s="27" t="str">
-        <x:v>成员 B / C</x:v>
+        <x:v>Android TFLite ReID 接入</x:v>
+      </x:c>
+      <x:c r="C13" s="19" t="str">
+        <x:v>成员 A</x:v>
       </x:c>
       <x:c r="D13" s="13" t="n">
-        <x:v>5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E13" s="13" t="n">
-        <x:v>7</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F13" s="13" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G13" s="37" t="str">
-        <x:v>测试</x:v>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="H13" s="12" t="str">
-        <x:v>手动遥控测试记录；形成第 1 周基础链路验收证据</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+        <x:v>Android ReID 可运行；Human Cart Simulator 中 ReID 字段正常，仍不作为单帧 FOLLOW 判决</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
         <x:v>T11</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>人物检测与目标初始化</x:v>
+        <x:v>诊断日志与 PC compare 闭环</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
         <x:v>成员 A</x:v>
       </x:c>
       <x:c r="D14" s="13" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E14" s="13" t="n">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F14" s="13" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G14" s="22" t="str">
-        <x:v>上位机</x:v>
+      <x:c r="G14" s="36" t="str">
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="H14" s="12" t="str">
-        <x:v>目标初始化可用；先在单人、受控场景下完成</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
+        <x:v>cartfollow_diagnostics；记录 frame/identity/events/gallery/crops，支持新旧数据对比</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
         <x:v>T12</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>单人直线跟随初版</x:v>
+        <x:v>track/bbox gate 与 relock 策略</x:v>
       </x:c>
       <x:c r="C15" s="19" t="str">
         <x:v>成员 A</x:v>
       </x:c>
       <x:c r="D15" s="13" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E15" s="13" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F15" s="13" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G15" s="22" t="str">
         <x:v>上位机</x:v>
       </x:c>
       <x:c r="H15" s="12" t="str">
-        <x:v>直线跟随初版；实现目标锁定与基础跟随控制</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="15" hidden="0" customHeight="1">
+        <x:v>目标轨迹与身份信念层；lockedTrack、suspectedTrack、ghost memory、空间支持门控已进入代码</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
         <x:v>T13</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>购物筐与载物平台结构改造</x:v>
-      </x:c>
-      <x:c r="C16" s="18" t="str">
-        <x:v>成员 C</x:v>
+        <x:v>底盘、麦轮与 AT8236 接线</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str">
+        <x:v>成员 B</x:v>
       </x:c>
       <x:c r="D16" s="13" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E16" s="13" t="n">
-        <x:v>14</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F16" s="13" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="G16" s="34" t="str">
-        <x:v>结构</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G16" s="30" t="str">
+        <x:v>硬件</x:v>
       </x:c>
       <x:c r="H16" s="12" t="str">
-        <x:v>购物筐结构完成；重点处理重心和安装稳固性</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="15" hidden="0" customHeight="1">
+        <x:v>实体底盘接线完成；四电机与 AT8236 完成连接，12V 电池搭载</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
         <x:v>T14</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>供电、驱动与负载稳定性调试</x:v>
+        <x:v>ESP32 串口与 WiFi 调控</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str">
         <x:v>成员 B</x:v>
       </x:c>
       <x:c r="D17" s="13" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E17" s="13" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F17" s="13" t="n">
         <x:v>5</x:v>
@@ -1156,163 +1156,163 @@
         <x:v>下位机</x:v>
       </x:c>
       <x:c r="H17" s="12" t="str">
-        <x:v>供电与驱动稳定；保证带载运行不掉压不过热</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
+        <x:v>CartESP32 WiFi 控制页；支持前后、转向、横移、停止和 host 控制命令</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
         <x:v>T15</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>跟随参数调节一轮</x:v>
-      </x:c>
-      <x:c r="C18" s="14" t="str">
-        <x:v>成员 A / C</x:v>
+        <x:v>轮向标定与限速保护</x:v>
+      </x:c>
+      <x:c r="C18" s="27" t="str">
+        <x:v>成员 B / C</x:v>
       </x:c>
       <x:c r="D18" s="13" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E18" s="13" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="F18" s="13" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G18" s="37" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G18" s="36" t="str">
         <x:v>测试</x:v>
       </x:c>
       <x:c r="H18" s="12" t="str">
-        <x:v>第一版参数表；调速度、距离、转向灵敏度</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
+        <x:v>轮向/速度测试记录；确认 M1-M4 对应关系、麦轮向量、低速限幅和松手停车</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
         <x:v>T16</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>急停按钮与停车执行链路</x:v>
-      </x:c>
-      <x:c r="C19" s="27" t="str">
-        <x:v>成员 B / C</x:v>
+        <x:v>通信超时与急停执行验证</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="str">
+        <x:v>成员 B</x:v>
       </x:c>
       <x:c r="D19" s="13" t="n">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E19" s="13" t="n">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F19" s="13" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G19" s="40" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G19" s="39" t="str">
         <x:v>安全</x:v>
       </x:c>
       <x:c r="H19" s="12" t="str">
-        <x:v>急停功能可用；未解除急停前不得再次启动</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
+        <x:v>失联停车记录；WiFi/host 指令超时、!S 停车和异常保护验证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
         <x:v>T17</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>通信超时停车保护</x:v>
-      </x:c>
-      <x:c r="C20" s="23" t="str">
-        <x:v>成员 B</x:v>
+        <x:v>手机支架、线束与电池固定</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
+        <x:v>成员 C / B</x:v>
       </x:c>
       <x:c r="D20" s="13" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="E20" s="13" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F20" s="13" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G20" s="40" t="str">
-        <x:v>安全</x:v>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G20" s="42" t="str">
+        <x:v>结构</x:v>
       </x:c>
       <x:c r="H20" s="12" t="str">
-        <x:v>断连保护可用；配合通信测试复验</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>结构固定初版；螺丝、铜柱、支架、转接线等补齐并安装</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
         <x:v>T18</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
-        <x:v>目标丢失安全搜索与停车</x:v>
-      </x:c>
-      <x:c r="C21" s="41" t="str">
-        <x:v>成员 A / B / C</x:v>
+        <x:v>购物筐/载物平台安装</x:v>
+      </x:c>
+      <x:c r="C21" s="18" t="str">
+        <x:v>成员 C</x:v>
       </x:c>
       <x:c r="D21" s="13" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="E21" s="13" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F21" s="13" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G21" s="40" t="str">
-        <x:v>安全</x:v>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G21" s="42" t="str">
+        <x:v>结构</x:v>
       </x:c>
       <x:c r="H21" s="12" t="str">
-        <x:v>LOST / SEARCH / STOP 联调完成；先取消前进，再短时原地搜索，超时停车</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
+        <x:v>载物平台初版；优先低重心、机械限位和轻载稳定演示</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
         <x:v>T19</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
-        <x:v>障碍停车集成</x:v>
-      </x:c>
-      <x:c r="C22" s="27" t="str">
-        <x:v>成员 C / B</x:v>
+        <x:v>Human Cart Simulator 手机复测</x:v>
+      </x:c>
+      <x:c r="C22" s="14" t="str">
+        <x:v>成员 A / C</x:v>
       </x:c>
       <x:c r="D22" s="13" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E22" s="13" t="n">
-        <x:v>19</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F22" s="13" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G22" s="40" t="str">
-        <x:v>安全</x:v>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G22" s="36" t="str">
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="H22" s="12" t="str">
-        <x:v>障碍停车可用；首版优先实现减速或停车</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
+        <x:v>四类场景复测数据；目标返回、遮挡恢复、干扰者进入、干扰者穿越</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
         <x:v>T20</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>系统联调一轮</x:v>
-      </x:c>
-      <x:c r="C23" s="41" t="str">
+        <x:v>极低速真实底盘联调门槛</x:v>
+      </x:c>
+      <x:c r="C23" s="43" t="str">
         <x:v>成员 A / B / C</x:v>
       </x:c>
       <x:c r="D23" s="13" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E23" s="13" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="F23" s="13" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G23" s="44" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G23" s="46" t="str">
         <x:v>联调</x:v>
       </x:c>
       <x:c r="H23" s="12" t="str">
-        <x:v>核心闭环初通；验证跟随与停车链路协同</x:v>
+        <x:v>联调准入结论；只有上位机复测和下位机停车保护稳定后才开放真实前进</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1320,103 +1320,103 @@
         <x:v>T21</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>中期材料与问题清单整理</x:v>
-      </x:c>
-      <x:c r="C24" s="45" t="str">
-        <x:v>成员 C / A / B</x:v>
+        <x:v>目标丢失与 LOCAL_SEARCH 联调</x:v>
+      </x:c>
+      <x:c r="C24" s="47" t="str">
+        <x:v>成员 A / B</x:v>
       </x:c>
       <x:c r="D24" s="13" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E24" s="13" t="n">
-        <x:v>18</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F24" s="13" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G24" s="17" t="str">
-        <x:v>项目规划</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G24" s="39" t="str">
+        <x:v>安全</x:v>
       </x:c>
       <x:c r="H24" s="12" t="str">
-        <x:v>中期汇报材料；整理已完成内容、问题和最后一周计划</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="15" hidden="0" customHeight="1">
+        <x:v>LOST/SEARCH/STOP 测试；先 motion_stop，再短时原地搜索，失败 hard STOP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
         <x:v>T22</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>转弯、停下与负载测试</x:v>
-      </x:c>
-      <x:c r="C25" s="45" t="str">
-        <x:v>成员 C / A / B</x:v>
+        <x:v>基础障碍停车/等待策略</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str">
+        <x:v>成员 A / C</x:v>
       </x:c>
       <x:c r="D25" s="13" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E25" s="13" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F25" s="13" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G25" s="37" t="str">
-        <x:v>测试</x:v>
+      <x:c r="G25" s="39" t="str">
+        <x:v>安全</x:v>
       </x:c>
       <x:c r="H25" s="12" t="str">
-        <x:v>测试记录补全；补足非直线路径和载物场景</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
+        <x:v>障碍处理测试记录；首版保守停车或等待，不做复杂 SLAM 绕障</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
         <x:v>T23</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>系统联调二轮与问题收敛</x:v>
-      </x:c>
-      <x:c r="C26" s="41" t="str">
-        <x:v>成员 A / B / C</x:v>
+        <x:v>负载、转弯与稳定性测试</x:v>
+      </x:c>
+      <x:c r="C26" s="27" t="str">
+        <x:v>成员 C / B</x:v>
       </x:c>
       <x:c r="D26" s="13" t="n">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E26" s="13" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="F26" s="13" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G26" s="44" t="str">
-        <x:v>联调</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G26" s="36" t="str">
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="H26" s="12" t="str">
-        <x:v>稳定版参数与流程；围绕最终演示脚本收敛问题</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
+        <x:v>1-3 kg 负载测试；验证结构松动、重心、转弯、急停与供电稳定性</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
         <x:v>T24</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
-        <x:v>演示视频录制与脚本固化</x:v>
-      </x:c>
-      <x:c r="C27" s="45" t="str">
-        <x:v>成员 C / A / B</x:v>
+        <x:v>系统联调与演示脚本固化</x:v>
+      </x:c>
+      <x:c r="C27" s="43" t="str">
+        <x:v>成员 A / B / C</x:v>
       </x:c>
       <x:c r="D27" s="13" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="E27" s="13" t="n">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F27" s="13" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G27" s="48" t="str">
-        <x:v>交付</x:v>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G27" s="46" t="str">
+        <x:v>联调</x:v>
       </x:c>
       <x:c r="H27" s="12" t="str">
-        <x:v>演示视频与脚本；保留分段演示与完整演示素材</x:v>
+        <x:v>稳定演示流程；固化手动遥控、目标确认、跟随、丢失搜索、停车演示</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1424,25 +1424,25 @@
         <x:v>T25</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>海报、PPT、总结报告收口</x:v>
-      </x:c>
-      <x:c r="C28" s="45" t="str">
+        <x:v>测试记录、视频与异常预案</x:v>
+      </x:c>
+      <x:c r="C28" s="48" t="str">
         <x:v>成员 C / A / B</x:v>
       </x:c>
       <x:c r="D28" s="13" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="E28" s="13" t="n">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F28" s="13" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G28" s="48" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G28" s="33" t="str">
         <x:v>交付</x:v>
       </x:c>
       <x:c r="H28" s="12" t="str">
-        <x:v>海报、PPT、总结报告；成员 C 主收口，A/B 提供技术内容</x:v>
+        <x:v>测试记录与演示视频；保留分段演示素材和失败降级预案</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
@@ -1450,25 +1450,51 @@
         <x:v>T26</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>最终彩排与现场预案确认</x:v>
-      </x:c>
-      <x:c r="C29" s="41" t="str">
+        <x:v>PPT、海报、报告收口</x:v>
+      </x:c>
+      <x:c r="C29" s="48" t="str">
+        <x:v>成员 C / A / B</x:v>
+      </x:c>
+      <x:c r="D29" s="13" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E29" s="13" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F29" s="13" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G29" s="33" t="str">
+        <x:v>交付</x:v>
+      </x:c>
+      <x:c r="H29" s="12" t="str">
+        <x:v>最终材料；A/B 提供技术内容，C 统一展示叙事</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A30" s="12" t="str">
+        <x:v>T27</x:v>
+      </x:c>
+      <x:c r="B30" s="12" t="str">
+        <x:v>最终彩排与参数冻结</x:v>
+      </x:c>
+      <x:c r="C30" s="43" t="str">
         <x:v>成员 A / B / C</x:v>
       </x:c>
-      <x:c r="D29" s="13" t="n">
+      <x:c r="D30" s="13" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E29" s="13" t="n">
+      <x:c r="E30" s="13" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="F29" s="13" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G29" s="48" t="str">
+      <x:c r="F30" s="13" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G30" s="33" t="str">
         <x:v>交付</x:v>
       </x:c>
-      <x:c r="H29" s="12" t="str">
-        <x:v>最终演示预案；保留保守参数、备件、电池和线材</x:v>
+      <x:c r="H30" s="12" t="str">
+        <x:v>最终演示预案；冻结保守参数、备份电池、备用线材和分段演示方案</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1584,13 +1610,13 @@
       <x:c r="S3" s="85" t="str">
         <x:v>第2周</x:v>
       </x:c>
-      <x:c r="T3" s="85" t="str">
+      <x:c r="T3" s="95" t="str">
         <x:v>第2周</x:v>
       </x:c>
       <x:c r="U3" s="58" t="str">
         <x:v>第3周</x:v>
       </x:c>
-      <x:c r="V3" s="95" t="str">
+      <x:c r="V3" s="58" t="str">
         <x:v>第3周</x:v>
       </x:c>
       <x:c r="W3" s="58" t="str">
@@ -1688,13 +1714,13 @@
       <x:c r="S4" s="86" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="T4" s="86" t="n">
+      <x:c r="T4" s="95" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="U4" s="60" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="V4" s="95" t="n">
+      <x:c r="V4" s="60" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="W4" s="60" t="n">
@@ -1774,13 +1800,13 @@
       <x:c r="S5" s="62" t="str">
         <x:v>第13天</x:v>
       </x:c>
-      <x:c r="T5" s="62" t="str">
+      <x:c r="T5" s="95" t="str">
         <x:v>第14天</x:v>
       </x:c>
       <x:c r="U5" s="62" t="str">
         <x:v>第15天</x:v>
       </x:c>
-      <x:c r="V5" s="95" t="str">
+      <x:c r="V5" s="62" t="str">
         <x:v>第16天</x:v>
       </x:c>
       <x:c r="W5" s="62" t="str">
@@ -1825,7 +1851,7 @@
         <x:v>T01</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>需求收口与关键指标确定</x:v>
+        <x:v>需求收口与首版边界确认</x:v>
       </x:c>
       <x:c r="C6" s="14" t="str">
         <x:v>成员 A / C</x:v>
@@ -1877,7 +1903,7 @@
         <x:v>T02</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>WBS、分工与物料清单初版</x:v>
+        <x:v>WBS、分工、BOM 初版</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
         <x:v>成员 C</x:v>
@@ -1931,35 +1957,33 @@
         <x:v>T03</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>方案 PPT 与汇报材料准备</x:v>
-      </x:c>
-      <x:c r="C8" s="14" t="str">
-        <x:v>成员 A / C</x:v>
-      </x:c>
-      <x:c r="D8" s="17" t="str">
-        <x:v>项目规划</x:v>
+        <x:v>OpenBot App 环境与源码梳理</x:v>
+      </x:c>
+      <x:c r="C8" s="19" t="str">
+        <x:v>成员 A</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="E8" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F8" s="13" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G8" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H8" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I8" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J8" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K8" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G8" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H8" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I8" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J8" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K8" s="84" t="str"/>
       <x:c r="L8" s="87" t="str"/>
       <x:c r="M8" s="87" t="str"/>
       <x:c r="N8" s="84" t="str"/>
@@ -1989,13 +2013,13 @@
         <x:v>T04</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>OpenBot App 环境搭建与编译</x:v>
-      </x:c>
-      <x:c r="C9" s="19" t="str">
-        <x:v>成员 A</x:v>
-      </x:c>
-      <x:c r="D9" s="22" t="str">
-        <x:v>上位机</x:v>
+        <x:v>下位机方案与 AT8236 风险分析</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="str">
+        <x:v>成员 B</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="str">
+        <x:v>下位机</x:v>
       </x:c>
       <x:c r="E9" s="13" t="n">
         <x:v>1</x:v>
@@ -2045,19 +2069,19 @@
         <x:v>T05</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>MCU 环境搭建与固件烧录</x:v>
-      </x:c>
-      <x:c r="C10" s="23" t="str">
-        <x:v>成员 B</x:v>
-      </x:c>
-      <x:c r="D10" s="26" t="str">
-        <x:v>下位机</x:v>
+        <x:v>底盘、电机、电池、驱动板采购</x:v>
+      </x:c>
+      <x:c r="C10" s="27" t="str">
+        <x:v>成员 B / C</x:v>
+      </x:c>
+      <x:c r="D10" s="30" t="str">
+        <x:v>硬件</x:v>
       </x:c>
       <x:c r="E10" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F10" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G10" s="80" t="n">
         <x:v>2</x:v>
@@ -2068,8 +2092,12 @@
       <x:c r="I10" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="J10" s="84" t="str"/>
-      <x:c r="K10" s="84" t="str"/>
+      <x:c r="J10" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K10" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="L10" s="87" t="str"/>
       <x:c r="M10" s="87" t="str"/>
       <x:c r="N10" s="84" t="str"/>
@@ -2099,35 +2127,37 @@
         <x:v>T06</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>底盘、电机、电源到货检查</x:v>
-      </x:c>
-      <x:c r="C11" s="27" t="str">
-        <x:v>成员 B / C</x:v>
-      </x:c>
-      <x:c r="D11" s="30" t="str">
-        <x:v>硬件</x:v>
+        <x:v>方案 PPT 与第 1 周材料</x:v>
+      </x:c>
+      <x:c r="C11" s="14" t="str">
+        <x:v>成员 A / C</x:v>
+      </x:c>
+      <x:c r="D11" s="33" t="str">
+        <x:v>交付</x:v>
       </x:c>
       <x:c r="E11" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F11" s="13" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G11" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H11" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="I11" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J11" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K11" s="84" t="str"/>
-      <x:c r="L11" s="87" t="str"/>
-      <x:c r="M11" s="87" t="str"/>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G11" s="84" t="str"/>
+      <x:c r="H11" s="84" t="str"/>
+      <x:c r="I11" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J11" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K11" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L11" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M11" s="78" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="N11" s="84" t="str"/>
       <x:c r="O11" s="84" t="str"/>
       <x:c r="P11" s="84" t="str"/>
@@ -2155,38 +2185,40 @@
         <x:v>T07</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>手机与下位机串口通信打通</x:v>
-      </x:c>
-      <x:c r="C12" s="31" t="str">
-        <x:v>成员 B / A</x:v>
-      </x:c>
-      <x:c r="D12" s="26" t="str">
-        <x:v>下位机</x:v>
+        <x:v>Human Cart Simulator 主流程</x:v>
+      </x:c>
+      <x:c r="C12" s="19" t="str">
+        <x:v>成员 A</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="E12" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F12" s="13" t="n">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G12" s="84" t="str"/>
       <x:c r="H12" s="84" t="str"/>
-      <x:c r="I12" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J12" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K12" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="I12" s="84" t="str"/>
+      <x:c r="J12" s="84" t="str"/>
+      <x:c r="K12" s="84" t="str"/>
       <x:c r="L12" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="M12" s="87" t="str"/>
-      <x:c r="N12" s="84" t="str"/>
-      <x:c r="O12" s="84" t="str"/>
-      <x:c r="P12" s="84" t="str"/>
+      <x:c r="M12" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N12" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O12" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P12" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="Q12" s="84" t="str"/>
       <x:c r="R12" s="84" t="str"/>
       <x:c r="S12" s="87" t="str"/>
@@ -2211,42 +2243,38 @@
         <x:v>T08</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>底盘装配与基础运动联调</x:v>
-      </x:c>
-      <x:c r="C13" s="23" t="str">
-        <x:v>成员 B</x:v>
-      </x:c>
-      <x:c r="D13" s="30" t="str">
-        <x:v>硬件</x:v>
+        <x:v>距离控制图像伺服</x:v>
+      </x:c>
+      <x:c r="C13" s="19" t="str">
+        <x:v>成员 A</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="E13" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F13" s="13" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G13" s="84" t="str"/>
       <x:c r="H13" s="84" t="str"/>
-      <x:c r="I13" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J13" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K13" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="L13" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="M13" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="N13" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O13" s="84" t="str"/>
-      <x:c r="P13" s="84" t="str"/>
+      <x:c r="I13" s="84" t="str"/>
+      <x:c r="J13" s="84" t="str"/>
+      <x:c r="K13" s="84" t="str"/>
+      <x:c r="L13" s="87" t="str"/>
+      <x:c r="M13" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N13" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O13" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P13" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="Q13" s="84" t="str"/>
       <x:c r="R13" s="84" t="str"/>
       <x:c r="S13" s="87" t="str"/>
@@ -2271,39 +2299,41 @@
         <x:v>T09</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>手机支架与视角固定</x:v>
-      </x:c>
-      <x:c r="C14" s="18" t="str">
-        <x:v>成员 C</x:v>
-      </x:c>
-      <x:c r="D14" s="34" t="str">
-        <x:v>结构</x:v>
+        <x:v>ReID PC 实验与 gallery 策略</x:v>
+      </x:c>
+      <x:c r="C14" s="19" t="str">
+        <x:v>成员 A</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="E14" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F14" s="13" t="n">
-        <x:v>6</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G14" s="84" t="str"/>
       <x:c r="H14" s="84" t="str"/>
-      <x:c r="I14" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J14" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K14" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L14" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M14" s="87" t="str"/>
-      <x:c r="N14" s="84" t="str"/>
-      <x:c r="O14" s="84" t="str"/>
-      <x:c r="P14" s="84" t="str"/>
-      <x:c r="Q14" s="84" t="str"/>
+      <x:c r="I14" s="84" t="str"/>
+      <x:c r="J14" s="84" t="str"/>
+      <x:c r="K14" s="84" t="str"/>
+      <x:c r="L14" s="87" t="str"/>
+      <x:c r="M14" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N14" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O14" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P14" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q14" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="R14" s="84" t="str"/>
       <x:c r="S14" s="87" t="str"/>
       <x:c r="T14" s="87" t="str"/>
@@ -2327,38 +2357,40 @@
         <x:v>T10</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>手动遥控测试与记录</x:v>
-      </x:c>
-      <x:c r="C15" s="27" t="str">
-        <x:v>成员 B / C</x:v>
-      </x:c>
-      <x:c r="D15" s="37" t="str">
-        <x:v>测试</x:v>
+        <x:v>Android TFLite ReID 接入</x:v>
+      </x:c>
+      <x:c r="C15" s="19" t="str">
+        <x:v>成员 A</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="str">
+        <x:v>上位机</x:v>
       </x:c>
       <x:c r="E15" s="13" t="n">
-        <x:v>5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F15" s="13" t="n">
-        <x:v>7</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G15" s="84" t="str"/>
       <x:c r="H15" s="84" t="str"/>
       <x:c r="I15" s="84" t="str"/>
       <x:c r="J15" s="84" t="str"/>
-      <x:c r="K15" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="L15" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="M15" s="78" t="n">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="K15" s="84" t="str"/>
+      <x:c r="L15" s="87" t="str"/>
+      <x:c r="M15" s="87" t="str"/>
       <x:c r="N15" s="84" t="str"/>
-      <x:c r="O15" s="84" t="str"/>
-      <x:c r="P15" s="84" t="str"/>
-      <x:c r="Q15" s="84" t="str"/>
-      <x:c r="R15" s="84" t="str"/>
+      <x:c r="O15" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P15" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Q15" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R15" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="S15" s="87" t="str"/>
       <x:c r="T15" s="87" t="str"/>
       <x:c r="U15" s="84" t="str"/>
@@ -2381,19 +2413,19 @@
         <x:v>T11</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>人物检测与目标初始化</x:v>
+        <x:v>诊断日志与 PC compare 闭环</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
         <x:v>成员 A</x:v>
       </x:c>
-      <x:c r="D16" s="22" t="str">
-        <x:v>上位机</x:v>
+      <x:c r="D16" s="36" t="str">
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E16" s="13" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F16" s="13" t="n">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G16" s="84" t="str"/>
       <x:c r="H16" s="84" t="str"/>
@@ -2402,20 +2434,20 @@
       <x:c r="K16" s="84" t="str"/>
       <x:c r="L16" s="87" t="str"/>
       <x:c r="M16" s="87" t="str"/>
-      <x:c r="N16" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="O16" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="P16" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="Q16" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="R16" s="84" t="str"/>
-      <x:c r="S16" s="87" t="str"/>
+      <x:c r="N16" s="84" t="str"/>
+      <x:c r="O16" s="84" t="str"/>
+      <x:c r="P16" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q16" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R16" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S16" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="T16" s="87" t="str"/>
       <x:c r="U16" s="84" t="str"/>
       <x:c r="V16" s="84" t="str"/>
@@ -2437,7 +2469,7 @@
         <x:v>T12</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>单人直线跟随初版</x:v>
+        <x:v>track/bbox gate 与 relock 策略</x:v>
       </x:c>
       <x:c r="C17" s="19" t="str">
         <x:v>成员 A</x:v>
@@ -2446,10 +2478,10 @@
         <x:v>上位机</x:v>
       </x:c>
       <x:c r="E17" s="13" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F17" s="13" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G17" s="84" t="str"/>
       <x:c r="H17" s="84" t="str"/>
@@ -2459,12 +2491,8 @@
       <x:c r="L17" s="87" t="str"/>
       <x:c r="M17" s="87" t="str"/>
       <x:c r="N17" s="84" t="str"/>
-      <x:c r="O17" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="P17" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="O17" s="84" t="str"/>
+      <x:c r="P17" s="84" t="str"/>
       <x:c r="Q17" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -2474,7 +2502,9 @@
       <x:c r="S17" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="T17" s="87" t="str"/>
+      <x:c r="T17" s="78" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="U17" s="84" t="str"/>
       <x:c r="V17" s="84" t="str"/>
       <x:c r="W17" s="84" t="str"/>
@@ -2495,19 +2525,19 @@
         <x:v>T13</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>购物筐与载物平台结构改造</x:v>
-      </x:c>
-      <x:c r="C18" s="18" t="str">
-        <x:v>成员 C</x:v>
-      </x:c>
-      <x:c r="D18" s="34" t="str">
-        <x:v>结构</x:v>
+        <x:v>底盘、麦轮与 AT8236 接线</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="str">
+        <x:v>成员 B</x:v>
+      </x:c>
+      <x:c r="D18" s="30" t="str">
+        <x:v>硬件</x:v>
       </x:c>
       <x:c r="E18" s="13" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="F18" s="13" t="n">
-        <x:v>14</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G18" s="84" t="str"/>
       <x:c r="H18" s="84" t="str"/>
@@ -2516,27 +2546,23 @@
       <x:c r="K18" s="84" t="str"/>
       <x:c r="L18" s="87" t="str"/>
       <x:c r="M18" s="87" t="str"/>
-      <x:c r="N18" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O18" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="P18" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Q18" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R18" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S18" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T18" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="N18" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O18" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P18" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Q18" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R18" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="S18" s="87" t="str"/>
+      <x:c r="T18" s="87" t="str"/>
       <x:c r="U18" s="84" t="str"/>
       <x:c r="V18" s="84" t="str"/>
       <x:c r="W18" s="84" t="str"/>
@@ -2557,7 +2583,7 @@
         <x:v>T14</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>供电、驱动与负载稳定性调试</x:v>
+        <x:v>ESP32 串口与 WiFi 调控</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str">
         <x:v>成员 B</x:v>
@@ -2566,10 +2592,10 @@
         <x:v>下位机</x:v>
       </x:c>
       <x:c r="E19" s="13" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F19" s="13" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G19" s="84" t="str"/>
       <x:c r="H19" s="84" t="str"/>
@@ -2578,9 +2604,7 @@
       <x:c r="K19" s="84" t="str"/>
       <x:c r="L19" s="87" t="str"/>
       <x:c r="M19" s="87" t="str"/>
-      <x:c r="N19" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="N19" s="84" t="str"/>
       <x:c r="O19" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -2593,7 +2617,9 @@
       <x:c r="R19" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="S19" s="87" t="str"/>
+      <x:c r="S19" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="T19" s="87" t="str"/>
       <x:c r="U19" s="84" t="str"/>
       <x:c r="V19" s="84" t="str"/>
@@ -2615,16 +2641,16 @@
         <x:v>T15</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>跟随参数调节一轮</x:v>
-      </x:c>
-      <x:c r="C20" s="14" t="str">
-        <x:v>成员 A / C</x:v>
-      </x:c>
-      <x:c r="D20" s="37" t="str">
+        <x:v>轮向标定与限速保护</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
+        <x:v>成员 B / C</x:v>
+      </x:c>
+      <x:c r="D20" s="36" t="str">
         <x:v>测试</x:v>
       </x:c>
       <x:c r="E20" s="13" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F20" s="13" t="n">
         <x:v>16</x:v>
@@ -2639,9 +2665,7 @@
       <x:c r="N20" s="84" t="str"/>
       <x:c r="O20" s="84" t="str"/>
       <x:c r="P20" s="84" t="str"/>
-      <x:c r="Q20" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="Q20" s="84" t="str"/>
       <x:c r="R20" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -2654,8 +2678,8 @@
       <x:c r="U20" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="V20" s="78" t="n">
-        <x:v>3</x:v>
+      <x:c r="V20" s="80" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="W20" s="84" t="str"/>
       <x:c r="X20" s="84" t="str"/>
@@ -2675,19 +2699,19 @@
         <x:v>T16</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
-        <x:v>急停按钮与停车执行链路</x:v>
-      </x:c>
-      <x:c r="C21" s="27" t="str">
-        <x:v>成员 B / C</x:v>
-      </x:c>
-      <x:c r="D21" s="40" t="str">
+        <x:v>通信超时与急停执行验证</x:v>
+      </x:c>
+      <x:c r="C21" s="23" t="str">
+        <x:v>成员 B</x:v>
+      </x:c>
+      <x:c r="D21" s="39" t="str">
         <x:v>安全</x:v>
       </x:c>
       <x:c r="E21" s="13" t="n">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F21" s="13" t="n">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G21" s="84" t="str"/>
       <x:c r="H21" s="84" t="str"/>
@@ -2698,15 +2722,9 @@
       <x:c r="M21" s="87" t="str"/>
       <x:c r="N21" s="84" t="str"/>
       <x:c r="O21" s="84" t="str"/>
-      <x:c r="P21" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="Q21" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="R21" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="P21" s="84" t="str"/>
+      <x:c r="Q21" s="84" t="str"/>
+      <x:c r="R21" s="84" t="str"/>
       <x:c r="S21" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -2716,8 +2734,12 @@
       <x:c r="U21" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="V21" s="84" t="str"/>
-      <x:c r="W21" s="84" t="str"/>
+      <x:c r="V21" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W21" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="X21" s="84" t="str"/>
       <x:c r="Y21" s="84" t="str"/>
       <x:c r="Z21" s="87" t="str"/>
@@ -2735,19 +2757,19 @@
         <x:v>T17</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
-        <x:v>通信超时停车保护</x:v>
-      </x:c>
-      <x:c r="C22" s="23" t="str">
-        <x:v>成员 B</x:v>
-      </x:c>
-      <x:c r="D22" s="40" t="str">
-        <x:v>安全</x:v>
+        <x:v>手机支架、线束与电池固定</x:v>
+      </x:c>
+      <x:c r="C22" s="27" t="str">
+        <x:v>成员 C / B</x:v>
+      </x:c>
+      <x:c r="D22" s="42" t="str">
+        <x:v>结构</x:v>
       </x:c>
       <x:c r="E22" s="13" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F22" s="13" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G22" s="84" t="str"/>
       <x:c r="H22" s="84" t="str"/>
@@ -2774,7 +2796,9 @@
       <x:c r="U22" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="V22" s="84" t="str"/>
+      <x:c r="V22" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="W22" s="84" t="str"/>
       <x:c r="X22" s="84" t="str"/>
       <x:c r="Y22" s="84" t="str"/>
@@ -2793,19 +2817,19 @@
         <x:v>T18</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>目标丢失安全搜索与停车</x:v>
-      </x:c>
-      <x:c r="C23" s="41" t="str">
-        <x:v>成员 A / B / C</x:v>
-      </x:c>
-      <x:c r="D23" s="40" t="str">
-        <x:v>安全</x:v>
+        <x:v>购物筐/载物平台安装</x:v>
+      </x:c>
+      <x:c r="C23" s="18" t="str">
+        <x:v>成员 C</x:v>
+      </x:c>
+      <x:c r="D23" s="42" t="str">
+        <x:v>结构</x:v>
       </x:c>
       <x:c r="E23" s="13" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="F23" s="13" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G23" s="84" t="str"/>
       <x:c r="H23" s="84" t="str"/>
@@ -2820,22 +2844,24 @@
       <x:c r="Q23" s="84" t="str"/>
       <x:c r="R23" s="84" t="str"/>
       <x:c r="S23" s="87" t="str"/>
-      <x:c r="T23" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="U23" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="V23" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="W23" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="X23" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="Y23" s="84" t="str"/>
+      <x:c r="T23" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U23" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V23" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W23" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X23" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y23" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="Z23" s="87" t="str"/>
       <x:c r="AA23" s="87" t="str"/>
       <x:c r="AB23" s="84" t="str"/>
@@ -2851,19 +2877,19 @@
         <x:v>T19</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>障碍停车集成</x:v>
-      </x:c>
-      <x:c r="C24" s="27" t="str">
-        <x:v>成员 C / B</x:v>
-      </x:c>
-      <x:c r="D24" s="40" t="str">
-        <x:v>安全</x:v>
+        <x:v>Human Cart Simulator 手机复测</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>成员 A / C</x:v>
+      </x:c>
+      <x:c r="D24" s="36" t="str">
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E24" s="13" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F24" s="13" t="n">
-        <x:v>19</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G24" s="84" t="str"/>
       <x:c r="H24" s="84" t="str"/>
@@ -2878,22 +2904,20 @@
       <x:c r="Q24" s="84" t="str"/>
       <x:c r="R24" s="84" t="str"/>
       <x:c r="S24" s="87" t="str"/>
-      <x:c r="T24" s="87" t="str"/>
-      <x:c r="U24" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="V24" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W24" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X24" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y24" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="T24" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U24" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="V24" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W24" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="X24" s="84" t="str"/>
+      <x:c r="Y24" s="84" t="str"/>
       <x:c r="Z24" s="87" t="str"/>
       <x:c r="AA24" s="87" t="str"/>
       <x:c r="AB24" s="84" t="str"/>
@@ -2909,16 +2933,16 @@
         <x:v>T20</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>系统联调一轮</x:v>
-      </x:c>
-      <x:c r="C25" s="41" t="str">
+        <x:v>极低速真实底盘联调门槛</x:v>
+      </x:c>
+      <x:c r="C25" s="43" t="str">
         <x:v>成员 A / B / C</x:v>
       </x:c>
-      <x:c r="D25" s="44" t="str">
+      <x:c r="D25" s="46" t="str">
         <x:v>联调</x:v>
       </x:c>
       <x:c r="E25" s="13" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F25" s="13" t="n">
         <x:v>20</x:v>
@@ -2938,9 +2962,7 @@
       <x:c r="S25" s="87" t="str"/>
       <x:c r="T25" s="87" t="str"/>
       <x:c r="U25" s="84" t="str"/>
-      <x:c r="V25" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="V25" s="84" t="str"/>
       <x:c r="W25" s="80" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -2967,19 +2989,19 @@
         <x:v>T21</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>中期材料与问题清单整理</x:v>
-      </x:c>
-      <x:c r="C26" s="45" t="str">
-        <x:v>成员 C / A / B</x:v>
-      </x:c>
-      <x:c r="D26" s="17" t="str">
-        <x:v>项目规划</x:v>
+        <x:v>目标丢失与 LOCAL_SEARCH 联调</x:v>
+      </x:c>
+      <x:c r="C26" s="47" t="str">
+        <x:v>成员 A / B</x:v>
+      </x:c>
+      <x:c r="D26" s="39" t="str">
+        <x:v>安全</x:v>
       </x:c>
       <x:c r="E26" s="13" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F26" s="13" t="n">
-        <x:v>18</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G26" s="84" t="str"/>
       <x:c r="H26" s="84" t="str"/>
@@ -2997,16 +3019,22 @@
       <x:c r="T26" s="87" t="str"/>
       <x:c r="U26" s="84" t="str"/>
       <x:c r="V26" s="84" t="str"/>
-      <x:c r="W26" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X26" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y26" s="84" t="str"/>
-      <x:c r="Z26" s="87" t="str"/>
-      <x:c r="AA26" s="87" t="str"/>
-      <x:c r="AB26" s="84" t="str"/>
+      <x:c r="W26" s="84" t="str"/>
+      <x:c r="X26" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Y26" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Z26" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AA26" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AB26" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="AC26" s="84" t="str"/>
       <x:c r="AD26" s="84" t="str"/>
       <x:c r="AE26" s="84" t="str"/>
@@ -3019,19 +3047,19 @@
         <x:v>T22</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
-        <x:v>转弯、停下与负载测试</x:v>
-      </x:c>
-      <x:c r="C27" s="45" t="str">
-        <x:v>成员 C / A / B</x:v>
-      </x:c>
-      <x:c r="D27" s="37" t="str">
-        <x:v>测试</x:v>
+        <x:v>基础障碍停车/等待策略</x:v>
+      </x:c>
+      <x:c r="C27" s="14" t="str">
+        <x:v>成员 A / C</x:v>
+      </x:c>
+      <x:c r="D27" s="39" t="str">
+        <x:v>安全</x:v>
       </x:c>
       <x:c r="E27" s="13" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F27" s="13" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G27" s="84" t="str"/>
       <x:c r="H27" s="84" t="str"/>
@@ -3050,9 +3078,7 @@
       <x:c r="U27" s="84" t="str"/>
       <x:c r="V27" s="84" t="str"/>
       <x:c r="W27" s="84" t="str"/>
-      <x:c r="X27" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="X27" s="84" t="str"/>
       <x:c r="Y27" s="79" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -3065,7 +3091,9 @@
       <x:c r="AB27" s="79" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AC27" s="84" t="str"/>
+      <x:c r="AC27" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="AD27" s="84" t="str"/>
       <x:c r="AE27" s="84" t="str"/>
       <x:c r="AF27" s="84" t="str"/>
@@ -3077,16 +3105,16 @@
         <x:v>T23</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>系统联调二轮与问题收敛</x:v>
-      </x:c>
-      <x:c r="C28" s="41" t="str">
-        <x:v>成员 A / B / C</x:v>
-      </x:c>
-      <x:c r="D28" s="44" t="str">
-        <x:v>联调</x:v>
+        <x:v>负载、转弯与稳定性测试</x:v>
+      </x:c>
+      <x:c r="C28" s="27" t="str">
+        <x:v>成员 C / B</x:v>
+      </x:c>
+      <x:c r="D28" s="36" t="str">
+        <x:v>测试</x:v>
       </x:c>
       <x:c r="E28" s="13" t="n">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F28" s="13" t="n">
         <x:v>24</x:v>
@@ -3110,18 +3138,20 @@
       <x:c r="W28" s="84" t="str"/>
       <x:c r="X28" s="84" t="str"/>
       <x:c r="Y28" s="84" t="str"/>
-      <x:c r="Z28" s="87" t="str"/>
-      <x:c r="AA28" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="AB28" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="AC28" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="AD28" s="80" t="n">
-        <x:v>2</x:v>
+      <x:c r="Z28" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AA28" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB28" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC28" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD28" s="79" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AE28" s="84" t="str"/>
       <x:c r="AF28" s="84" t="str"/>
@@ -3133,19 +3163,19 @@
         <x:v>T24</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>演示视频录制与脚本固化</x:v>
-      </x:c>
-      <x:c r="C29" s="45" t="str">
-        <x:v>成员 C / A / B</x:v>
-      </x:c>
-      <x:c r="D29" s="48" t="str">
-        <x:v>交付</x:v>
+        <x:v>系统联调与演示脚本固化</x:v>
+      </x:c>
+      <x:c r="C29" s="43" t="str">
+        <x:v>成员 A / B / C</x:v>
+      </x:c>
+      <x:c r="D29" s="46" t="str">
+        <x:v>联调</x:v>
       </x:c>
       <x:c r="E29" s="13" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="F29" s="13" t="n">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G29" s="84" t="str"/>
       <x:c r="H29" s="84" t="str"/>
@@ -3168,21 +3198,19 @@
       <x:c r="Y29" s="84" t="str"/>
       <x:c r="Z29" s="87" t="str"/>
       <x:c r="AA29" s="87" t="str"/>
-      <x:c r="AB29" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AC29" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AD29" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE29" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF29" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="AB29" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AC29" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AD29" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AE29" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AF29" s="84" t="str"/>
       <x:c r="AG29" s="87" t="str"/>
       <x:c r="AH29" s="87" t="str"/>
     </x:row>
@@ -3191,19 +3219,19 @@
         <x:v>T25</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>海报、PPT、总结报告收口</x:v>
-      </x:c>
-      <x:c r="C30" s="45" t="str">
+        <x:v>测试记录、视频与异常预案</x:v>
+      </x:c>
+      <x:c r="C30" s="48" t="str">
         <x:v>成员 C / A / B</x:v>
       </x:c>
-      <x:c r="D30" s="48" t="str">
+      <x:c r="D30" s="33" t="str">
         <x:v>交付</x:v>
       </x:c>
       <x:c r="E30" s="13" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="F30" s="13" t="n">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G30" s="84" t="str"/>
       <x:c r="H30" s="84" t="str"/>
@@ -3239,9 +3267,7 @@
       <x:c r="AF30" s="79" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AG30" s="79" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="AG30" s="87" t="str"/>
       <x:c r="AH30" s="87" t="str"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
@@ -3249,19 +3275,19 @@
         <x:v>T26</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>最终彩排与现场预案确认</x:v>
-      </x:c>
-      <x:c r="C31" s="41" t="str">
-        <x:v>成员 A / B / C</x:v>
-      </x:c>
-      <x:c r="D31" s="48" t="str">
+        <x:v>PPT、海报、报告收口</x:v>
+      </x:c>
+      <x:c r="C31" s="48" t="str">
+        <x:v>成员 C / A / B</x:v>
+      </x:c>
+      <x:c r="D31" s="33" t="str">
         <x:v>交付</x:v>
       </x:c>
       <x:c r="E31" s="13" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F31" s="13" t="n">
         <x:v>27</x:v>
-      </x:c>
-      <x:c r="F31" s="13" t="n">
-        <x:v>28</x:v>
       </x:c>
       <x:c r="G31" s="84" t="str"/>
       <x:c r="H31" s="84" t="str"/>
@@ -3286,46 +3312,91 @@
       <x:c r="AA31" s="87" t="str"/>
       <x:c r="AB31" s="84" t="str"/>
       <x:c r="AC31" s="84" t="str"/>
-      <x:c r="AD31" s="84" t="str"/>
-      <x:c r="AE31" s="84" t="str"/>
-      <x:c r="AF31" s="84" t="str"/>
-      <x:c r="AG31" s="80" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="AH31" s="78" t="n">
+      <x:c r="AD31" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE31" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF31" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG31" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH31" s="87" t="str"/>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="12" t="str">
+        <x:v>T27</x:v>
+      </x:c>
+      <x:c r="B32" s="12" t="str">
+        <x:v>最终彩排与参数冻结</x:v>
+      </x:c>
+      <x:c r="C32" s="43" t="str">
+        <x:v>成员 A / B / C</x:v>
+      </x:c>
+      <x:c r="D32" s="33" t="str">
+        <x:v>交付</x:v>
+      </x:c>
+      <x:c r="E32" s="13" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F32" s="13" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G32" s="84" t="str"/>
+      <x:c r="H32" s="84" t="str"/>
+      <x:c r="I32" s="84" t="str"/>
+      <x:c r="J32" s="84" t="str"/>
+      <x:c r="K32" s="84" t="str"/>
+      <x:c r="L32" s="87" t="str"/>
+      <x:c r="M32" s="87" t="str"/>
+      <x:c r="N32" s="84" t="str"/>
+      <x:c r="O32" s="84" t="str"/>
+      <x:c r="P32" s="84" t="str"/>
+      <x:c r="Q32" s="84" t="str"/>
+      <x:c r="R32" s="84" t="str"/>
+      <x:c r="S32" s="87" t="str"/>
+      <x:c r="T32" s="87" t="str"/>
+      <x:c r="U32" s="84" t="str"/>
+      <x:c r="V32" s="84" t="str"/>
+      <x:c r="W32" s="84" t="str"/>
+      <x:c r="X32" s="84" t="str"/>
+      <x:c r="Y32" s="84" t="str"/>
+      <x:c r="Z32" s="87" t="str"/>
+      <x:c r="AA32" s="87" t="str"/>
+      <x:c r="AB32" s="84" t="str"/>
+      <x:c r="AC32" s="84" t="str"/>
+      <x:c r="AD32" s="84" t="str"/>
+      <x:c r="AE32" s="84" t="str"/>
+      <x:c r="AF32" s="84" t="str"/>
+      <x:c r="AG32" s="80" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AH32" s="78" t="n">
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A34" s="98" t="str">
+    <x:row r="35" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A35" s="98" t="str">
         <x:v>说明：本甘特图使用第 1 天至第 28 天的相对排期，不绑定自然日。蓝色条表示普通计划任务，橙色条表示关键路径任务，红色节点表示“不完成则后续无法开展”的里程碑节点，浅灰底用于标识每周后两天的节奏参考。</x:v>
       </x:c>
-      <x:c r="B34" s="98"/>
-      <x:c r="C34" s="98"/>
-      <x:c r="D34" s="98"/>
-      <x:c r="E34" s="98"/>
-      <x:c r="F34" s="98"/>
-    </x:row>
-    <x:row r="35" ht="79.19999694824219" hidden="0" customHeight="1">
-      <x:c r="A35" s="100" t="str">
-        <x:v>里程碑</x:v>
-      </x:c>
-      <x:c r="B35" s="103" t="str">
-        <x:v>M1</x:v>
-      </x:c>
-      <x:c r="C35" s="99" t="str">
-        <x:v>基础链路跑通：若 Week 1 前未跑通手动遥控与基础链路，后续自主跟随与安全联调无法开展。</x:v>
-      </x:c>
+      <x:c r="B35" s="98"/>
+      <x:c r="C35" s="98"/>
+      <x:c r="D35" s="98"/>
+      <x:c r="E35" s="98"/>
+      <x:c r="F35" s="98"/>
     </x:row>
     <x:row r="36" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A36" s="100" t="str">
         <x:v>里程碑</x:v>
       </x:c>
       <x:c r="B36" s="103" t="str">
-        <x:v>M2</x:v>
+        <x:v>M1</x:v>
       </x:c>
       <x:c r="C36" s="99" t="str">
-        <x:v>自主跟随初版完成：若目标初始化、直线跟随与首轮参数调节未完成，后续安全策略和系统联调无法开展。</x:v>
+        <x:v>需求与基础方案收口：第 1 周完成需求、WBS、BOM、OpenBot/下位机方案分析和阶段材料。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="79.19999694824219" hidden="0" customHeight="1">
@@ -3333,61 +3404,72 @@
         <x:v>里程碑</x:v>
       </x:c>
       <x:c r="B37" s="103" t="str">
-        <x:v>M3</x:v>
+        <x:v>M2</x:v>
       </x:c>
       <x:c r="C37" s="99" t="str">
-        <x:v>安全闭环联调完成：若急停、失联停车、目标丢失与系统联调未完成，后续展示录制和最终交付无法开展。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="66" hidden="0" customHeight="1">
+        <x:v>上位机策略闭环完成：Human Cart Simulator、ReID、诊断日志和 track/bbox gate 形成可复盘闭环。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A38" s="100" t="str">
         <x:v>里程碑</x:v>
       </x:c>
       <x:c r="B38" s="103" t="str">
+        <x:v>M3</x:v>
+      </x:c>
+      <x:c r="C38" s="99" t="str">
+        <x:v>真实底盘联调准入：ESP32/AT8236、轮向标定、通信超时停车、结构固定和上位机复测均达到低速联调门槛。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A39" s="100" t="str">
+        <x:v>里程碑</x:v>
+      </x:c>
+      <x:c r="B39" s="103" t="str">
         <x:v>M4</x:v>
       </x:c>
-      <x:c r="C38" s="99" t="str">
-        <x:v>最终展示闭环完成：若最终彩排与现场预案未完成，课程展示和材料收口无法按计划交付。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39"/>
-    <x:row r="40" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A40" s="99" t="str">
-        <x:v>并行主线</x:v>
-      </x:c>
-      <x:c r="B40" s="99" t="str">
-        <x:v>成员 A</x:v>
-      </x:c>
-      <x:c r="C40" s="99" t="str">
-        <x:v>OpenBot App、人物检测、目标锁定、跟随参数调节</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="C39" s="99" t="str">
+        <x:v>最终展示闭环完成：完成最终彩排、参数冻结、材料收口和现场预案。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40"/>
+    <x:row r="41" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A41" s="99" t="str">
         <x:v>并行主线</x:v>
       </x:c>
       <x:c r="B41" s="99" t="str">
-        <x:v>成员 B</x:v>
+        <x:v>成员 A</x:v>
       </x:c>
       <x:c r="C41" s="99" t="str">
-        <x:v>MCU、通信、电机驱动、供电与急停执行</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>OpenBot App、人物检测、目标锁定、跟随参数调节</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A42" s="99" t="str">
         <x:v>并行主线</x:v>
       </x:c>
       <x:c r="B42" s="99" t="str">
+        <x:v>成员 B</x:v>
+      </x:c>
+      <x:c r="C42" s="99" t="str">
+        <x:v>MCU、通信、电机驱动、供电与急停执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A43" s="99" t="str">
+        <x:v>并行主线</x:v>
+      </x:c>
+      <x:c r="B43" s="99" t="str">
         <x:v>成员 C</x:v>
       </x:c>
-      <x:c r="C42" s="99" t="str">
+      <x:c r="C43" s="99" t="str">
         <x:v>结构改造、安全测试、视频记录与材料收口</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:AH1"/>
-    <x:mergeCell ref="A34:F34"/>
+    <x:mergeCell ref="A35:F35"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>